<commit_message>
Zone HTML: option counts in every filter; poverty and unemployment range filters with descriptors
Bands (editable in zone_config.py) are named relative to the national rates
(P0 March 2025 8.47%, TPT August 2025 4.85%); every value maps to one band.
xlsx gains Poverty band (v2) and Unemployment band (v2) columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015fqtP2mhnw4ZyW8UgLq13n
</commit_message>
<xml_diff>
--- a/indonesia-higher-ed/zone/output/priority_zone.xlsx
+++ b/indonesia-higher-ed/zone/output/priority_zone.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority zone" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priority zone'!$A$1:$Z$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priority zone'!$A$1:$AB$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z71"/>
+  <dimension ref="A1:AB71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,6 +553,16 @@
           <t>Changed</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Poverty band (v2)</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Unemployment band (v2)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -667,6 +677,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -781,6 +801,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -895,6 +925,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1009,6 +1049,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1123,6 +1173,16 @@
           <t>Poverty</t>
         </is>
       </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1237,6 +1297,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1351,6 +1421,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1469,6 +1549,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1583,6 +1673,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1697,6 +1797,16 @@
           <t>Swim; Poverty</t>
         </is>
       </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1811,6 +1921,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1929,6 +2049,16 @@
           <t>Swim; Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2047,6 +2177,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2161,6 +2301,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2275,6 +2425,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2389,6 +2549,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2503,6 +2673,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2617,6 +2797,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2735,6 +2925,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2849,6 +3049,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2967,6 +3177,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3081,6 +3301,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3195,6 +3425,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3309,6 +3549,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3425,6 +3675,16 @@
           <t>Safety; Unemployment</t>
         </is>
       </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3539,6 +3799,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3653,6 +3923,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3771,6 +4051,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3885,6 +4175,16 @@
           <t>Swim; Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3999,6 +4299,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4113,6 +4423,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4227,6 +4547,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4341,6 +4671,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4455,6 +4795,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4569,6 +4919,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4683,6 +5043,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4797,6 +5167,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4911,6 +5291,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5025,6 +5415,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5143,6 +5543,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5261,6 +5671,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5375,6 +5795,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5489,6 +5919,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5603,6 +6043,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5717,6 +6167,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5831,6 +6291,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5945,6 +6415,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6059,6 +6539,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6173,6 +6663,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6287,6 +6787,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6401,6 +6911,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6515,6 +7035,16 @@
           <t>Poverty</t>
         </is>
       </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6633,6 +7163,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6747,6 +7287,16 @@
           <t>Swim</t>
         </is>
       </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6861,6 +7411,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB56" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6975,6 +7535,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>Above national (10-13%)</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7089,6 +7659,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>High (&gt;=13%)</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7203,6 +7783,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>Below national (3-4.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7317,6 +7907,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7431,6 +8031,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA61" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7545,6 +8155,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>High (&gt;=7%)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7659,6 +8279,16 @@
           <t>Poverty</t>
         </is>
       </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>Near national (8-10%)</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7773,6 +8403,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>Very low (&lt;3%)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7891,6 +8531,16 @@
           <t>Poverty</t>
         </is>
       </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8005,6 +8655,16 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA66" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8119,6 +8779,16 @@
           <t>Safety; Poverty</t>
         </is>
       </c>
+      <c r="AA67" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8233,6 +8903,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA68" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8347,6 +9027,16 @@
           <t>Swim; Safety</t>
         </is>
       </c>
+      <c r="AA69" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB69" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -8461,6 +9151,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="AA70" t="inlineStr">
+        <is>
+          <t>Very low (&lt;5%)</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr">
+        <is>
+          <t>Near national (4.5-5.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8575,9 +9275,19 @@
           <t>Safety</t>
         </is>
       </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t>Below national (5-8%)</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr">
+        <is>
+          <t>Above national (5.5-7%)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z71"/>
+  <autoFilter ref="A1:AB71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>